<commit_message>
Add email column and more phone/address details to Karnataka leads
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GH7UaoDJSnD8fV4SJkmson
</commit_message>
<xml_diff>
--- a/karnataka_herbalife_leads.xlsx
+++ b/karnataka_herbalife_leads.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$L$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$M$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -454,12 +454,13 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,25 +501,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Email (public listing)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Pitch angle</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Contacted on</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -558,19 +564,20 @@
           <t>+91 80 4965 2381</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1172</t>
         </is>
@@ -610,19 +617,20 @@
           <t>+91 81053 12345</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://magicpin.in/blog/gyms-in-bangalore</t>
         </is>
@@ -662,19 +670,20 @@
           <t>+91 98458 45740</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/637</t>
         </is>
@@ -709,20 +718,25 @@
           <t>1st Floor, No 52/3, Ranka Colony Rd, next to Epitome Crowne Apt, Bilekahalli, Bengaluru 560076</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1207</t>
         </is>
@@ -757,20 +771,25 @@
           <t>No. 126, Chabria Square, Kengal Hanumanthaiah Rd, Srinivas Colony, Sudhama Nagar, Bengaluru 560027</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/443</t>
         </is>
@@ -805,20 +824,25 @@
           <t>28, 1st Cross, Ramaiah Layout, Kammanahalli Main Rd, opp. St Charles School, Bengaluru 560084</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/660</t>
         </is>
@@ -853,20 +877,25 @@
           <t>Millennium Avenue, 16/1, 9th Main Rd, opp. Thaja Cake, Arehalli, Uttarahalli, Bengaluru 560061</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/930</t>
         </is>
@@ -901,20 +930,25 @@
           <t>2nd Floor, KK Plaza, 150, 80 Feet Rd, 1st Phase Girinagar, Banashankari, Bengaluru 560085</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/718</t>
         </is>
@@ -949,20 +983,25 @@
           <t>20th L Cross Rd, near VRR Homes, Gowda Muniswamy Garden, Ejipura, Bengaluru 560047</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/579</t>
         </is>
@@ -997,20 +1036,25 @@
           <t>Gear Road, Sarjapur-Marathahalli Rd, Carmelaram, Doddakannelli, Bengaluru 560035</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/325</t>
         </is>
@@ -1045,20 +1089,25 @@
           <t>Kamadhenu Nagar, B Narayanapura, Mahadevapura, Bengaluru 560016</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1091</t>
         </is>
@@ -1093,20 +1142,25 @@
           <t>Varthur Main Rd, opp. Jagriti Renaissance Apartment, Ramagondanahalli, Whitefield, Bengaluru 560066</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1162</t>
         </is>
@@ -1141,20 +1195,25 @@
           <t>Immadihalli Main Rd, Sathya Sai Layout, Whitefield, Bengaluru 560066</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1123</t>
         </is>
@@ -1189,20 +1248,25 @@
           <t>No 31/1 242/211, 1st Floor, next to Shilpitha Sunflower Apt, Borewell Rd, Nallurhalli, Whitefield, Bengaluru 560066</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1136</t>
         </is>
@@ -1237,20 +1301,25 @@
           <t>Borewell Rd, Phase 2, Dodsworth Layout, Whitefield, Bengaluru 560066</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/5866</t>
         </is>
@@ -1285,20 +1354,25 @@
           <t>2nd Floor, SLN Complex, near Shivakuntamma Temple, Immadihalli Main Rd, opp. NVT Life Square, Whitefield, Bengaluru 560066</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/1139</t>
         </is>
@@ -1338,19 +1412,20 @@
           <t>+91 98447 45185</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://www.cure.fit/cult/cult-pass/bangalore/GymX-Marathahalli/81</t>
         </is>
@@ -1390,19 +1465,20 @@
           <t>+91 90354 24322</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://magicpin.com/blog/category/fitness/best-yoga-classes-bangalore</t>
         </is>
@@ -1442,19 +1518,20 @@
           <t>+91 90354 24333</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://magicpin.com/blog/category/fitness/best-yoga-classes-bangalore</t>
         </is>
@@ -1494,19 +1571,20 @@
           <t>+91 90354 24333</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>https://lbb.in/places/Aayana-Yoga-Academy-whitefield-89e871</t>
         </is>
@@ -1541,20 +1619,25 @@
           <t>No.19, 3rd Floor, Aloka Mansion, 10th B Main Rd, Jayanagar 1st Block, Bengaluru 560011</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/2564</t>
         </is>
@@ -1589,20 +1672,29 @@
           <t>951, 36th Cross, 10th Main Rd, behind BSNL Exchange, 4th Block, Jayanagar, Bengaluru 560041</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
+          <t>see rashtrotthana.org</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/2354</t>
         </is>
@@ -1637,20 +1729,25 @@
           <t>Ground Floor, 114, 1st Cross Rd, KHB Colony, 6th Block, Koramangala, Bengaluru 560095</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/2494</t>
         </is>
@@ -1685,20 +1782,25 @@
           <t>3rd Floor, 80 Feet Rd, 4th Block, Koramangala, Bengaluru 560047</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/2984</t>
         </is>
@@ -1738,19 +1840,20 @@
           <t>+91 80 4446 4736</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/addo-supplement-store</t>
         </is>
@@ -1790,19 +1893,20 @@
           <t>+91 80 4572 9810</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/hits-enterprise</t>
         </is>
@@ -1842,19 +1946,20 @@
           <t>+91 80 4781 0046</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/abhirami-enterprises</t>
         </is>
@@ -1894,19 +1999,20 @@
           <t>+91 80 4446 0148</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/fitbros</t>
         </is>
@@ -1946,19 +2052,20 @@
           <t>+91 80 4456 6518</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/proteinshoppebengaluru</t>
         </is>
@@ -1998,19 +2105,20 @@
           <t>+91 80 4446 4726</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Owner and walk-in customers are fitness buyers. Pitch the owner as a personal customer or a business-opportunity prospect (not as a stockist, see Read Me).</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>https://m.indiamart.com/body-fittness</t>
         </is>
@@ -2045,20 +2153,29 @@
           <t>HCS Complex, Main Borewell Rd, 3rd Cross Rd, Whitefield, Bengaluru</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
           <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>https://organicmandya.com/pages/bangalore/whitefield</t>
         </is>
@@ -2093,20 +2210,29 @@
           <t>Sampige Rd, Vyalikaval, Kodandarampura, Malleshwaram, Bengaluru</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
           <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>https://organicmandya.com/pages/bangalore/malleshwaram</t>
         </is>
@@ -2141,20 +2267,29 @@
           <t>Bysani Enclave, Vanivilas Rd, near SLV Corner, Gandhi Bazaar, Bengaluru</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
           <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>https://organicmandya.com/pages/bangalore/basavanagudi</t>
         </is>
@@ -2189,20 +2324,29 @@
           <t>Ground Floor, 74, Naseer Pride, MM Road, Frazer Town, Bengaluru</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
           <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>https://organicmandya.com/pages/bangalore/frazertown</t>
         </is>
@@ -2237,20 +2381,29 @@
           <t>55, Yelenahalli Main Rd, Akshayanagar, Begur Hobli, Bengaluru</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
           <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>https://organicmandya.com/pages/bangalore/aksahyanagar</t>
         </is>
@@ -2282,23 +2435,32 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Magrath Rd, near Brigade Rd, Bengaluru</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
+          <t>Magrath Rd, Ashok Nagar, Bengaluru 560025</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>+91 80 4069 8857 / +91 80500 40101</t>
+        </is>
+      </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
+          <t>customerservice@garudamall.net</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>https://travel.sygic.com/en/poi/garuda-mall-poi:33665</t>
         </is>
@@ -2330,23 +2492,32 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Vittal Mallya Rd, Bengaluru</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
+          <t>#24, Vittal Mallya Rd, Bengaluru 560001</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>+91 96867 19002 (The Collection @ UB City)</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
+          <t>thecollectionubcity@gmail.com</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>https://besttime.app/app/India/Bangalore/shopping?page=1</t>
         </is>
@@ -2378,23 +2549,28 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Bannerghatta Rd, Bengaluru</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr">
+          <t>22, Bannerghatta Rd, Sarakki Industrial Layout, JP Nagar 3rd Phase, Bengaluru 560076</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>https://besttime.app/app/India/Bangalore/shopping?page=1</t>
         </is>
@@ -2429,20 +2605,25 @@
           <t>Kanakapura Rd, Bengaluru</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>https://besttime.app/app/India/Bangalore/shopping?page=1</t>
         </is>
@@ -2477,20 +2658,25 @@
           <t>154/B Pragathi Plaza, 1st Floor, Nandhi Circle, Dattagalli, BEML Layout 2nd Stage, RR Nagar, Mysuru 570033</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/12609</t>
         </is>
@@ -2525,20 +2711,25 @@
           <t>KD Circle, Manchegowdana Koppalu, Vijayanagar 2nd Stage, Mysuru 570017</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/listing/12667</t>
         </is>
@@ -2578,19 +2769,20 @@
           <t>+91 821 234 2705</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>https://in.worldorgs.com/catalog/mysuru/gym/flex-city</t>
         </is>
@@ -2625,20 +2817,25 @@
           <t>C&amp;D Block, 1527, Anikethana Rd, Kuvempu Nagara, Mysuru 570023</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/listing/141727</t>
         </is>
@@ -2670,23 +2867,28 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Kuvempunagar, Mysuru (get exact address on Google Maps)</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
+          <t>464, Udayaravi Rd, E&amp;F Block, Kuvempu Nagara, Mysuru 570023</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/mysore/in/kuvempunagara</t>
         </is>
@@ -2721,20 +2923,25 @@
           <t>Kuvempunagar, Mysuru (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/mysore/in/kuvempunagara</t>
         </is>
@@ -2769,20 +2976,25 @@
           <t>Kuvempunagar, Mysuru (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>https://discover.lyfskills.com/gyms/mysore/in/kuvempunagara</t>
         </is>
@@ -2814,23 +3026,28 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Mysuru (largest mall in Mysuru)</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr">
+          <t>No. 8 &amp; N-5, Hyderali Rd, Nazarbad Mohalla, Mysuru 570010</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>+91 821 230 0402</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Nexus_Centre_City_Mall</t>
         </is>
@@ -2862,23 +3079,28 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Next to Mysore Racecourse, Mysuru</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr">
+          <t>No. C-1, MG Road, Indira Nagar, Nazarbad Mohalla, Mysuru 570010</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>+91 821 428 3555</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Mall_of_Mysore</t>
         </is>
@@ -2918,19 +3140,20 @@
           <t>+91 95351 22680</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>https://yappe.in/karnataka/hubballi/shadozzz-gym/1639689</t>
         </is>
@@ -2970,19 +3193,20 @@
           <t>+91 96069 82205</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>https://yappe.in/karnataka/hubballi/ifitness/1639677</t>
         </is>
@@ -3022,19 +3246,20 @@
           <t>+91 94481 88404</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>https://yappe.in/karnataka/hubballi/paramount-gym/1639695</t>
         </is>
@@ -3069,20 +3294,25 @@
           <t>Chennamma Circle, Hubballi</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/studio/muscle-factory-gyms-chennamma-circle</t>
         </is>
@@ -3117,20 +3347,25 @@
           <t>Vishweshwar Nagar, Hubballi</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/studio/muscle-factory-gyms-vishweshwar-nagar</t>
         </is>
@@ -3162,23 +3397,28 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Gokul Industrial Estate, Gokul Rd, Hubballi 580030 (largest mall in North Karnataka)</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr">
+          <t>CTS No 4784/B, 2nd Cross, Gokul Rd, Chaitanya Nagar, Hubballi 580030</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>+91 80 2235 2828 (Bengaluru code - verify)</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Urban_Oasis_Mall</t>
         </is>
@@ -3218,19 +3458,20 @@
           <t>+91 90368 77525</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr">
         <is>
           <t>https://yappe.in/karnataka/belagavi/x-fit-the-training-ground/783685</t>
         </is>
@@ -3265,20 +3506,25 @@
           <t>Tilakwadi, Belagavi (has a ladies-only section)</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr">
         <is>
           <t>https://bodyfitgarage8.odoo.com/blog/gym-fitness-centre-10/gym-fitness-centre-8</t>
         </is>
@@ -3309,20 +3555,25 @@
           <t>Belagavi (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr">
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/blog/best-and-top-gyms-in-belagavi</t>
         </is>
@@ -3353,20 +3604,25 @@
           <t>Belagavi (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/blog/best-and-top-gyms-in-belagavi</t>
         </is>
@@ -3397,20 +3653,25 @@
           <t>Belagavi (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/blog/best-and-top-gyms-in-belagavi</t>
         </is>
@@ -3441,20 +3702,25 @@
           <t>Belagavi (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr">
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/blog/best-and-top-gyms-in-belagavi</t>
         </is>
@@ -3485,20 +3751,25 @@
           <t>Belagavi (get exact address on Google Maps)</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr">
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/blog/best-and-top-gyms-in-belagavi</t>
         </is>
@@ -3533,20 +3804,25 @@
           <t>Maratha Colony, Belagavi</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr">
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/activities/gym/belagavi</t>
         </is>
@@ -3581,20 +3857,25 @@
           <t>Kavoor, Mangaluru</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/mangaluru/fitness-centers</t>
         </is>
@@ -3629,20 +3910,25 @@
           <t>Bendoor, Mangaluru</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K65" s="2" t="inlineStr"/>
-      <c r="L65" s="2" t="inlineStr">
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/mangaluru/fitness-centers</t>
         </is>
@@ -3677,20 +3963,25 @@
           <t>Valencia, Mangaluru</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/mangaluru/fitness-centers</t>
         </is>
@@ -3725,20 +4016,25 @@
           <t>Kadri / Kulshekar, Mangaluru</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K67" s="2" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr">
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
         <is>
           <t>https://rentechdigital.com/smartscraper/business-report-details/india/karnataka/list-of-gyms-in-mangalore</t>
         </is>
@@ -3773,20 +4069,25 @@
           <t>Bejai, Mangaluru</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K68" s="2" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/mangaluru/bejai/fitness-centers</t>
         </is>
@@ -3821,20 +4122,25 @@
           <t>Ground Floor, Anna Vista, next to Car Decor, Mallikatte, Kadri, Mangaluru 575002</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>Customers buying home-gym equipment are fitness buyers. Ask the owner about a referral tie-up.</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
         <is>
           <t>https://www.bikes4sale.in/new-bike-showrooms/dealer/coppernicus/karnataka/mangalore/16285/jyothi-cycle-fitness</t>
         </is>
@@ -3869,20 +4175,25 @@
           <t>Deralakatte, Belma Village, opp. KSHEMA, Mangaluru 575018</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
         <is>
           <t>https://www.urbanpro.com/mangalore/satwa-yoga-therapy-centre-mangalanthi/34618626</t>
         </is>
@@ -3914,23 +4225,28 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Pandeshwar, Mangaluru (largest mall in Mangaluru)</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr">
+          <t>Mangaladevi Rd, Pandeshwar, Mangaluru</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr">
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Pandeshwar</t>
         </is>
@@ -3958,23 +4274,28 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Mangaluru</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr">
+          <t>KS Rao Rd, Hampankatta, Mangaluru 575001 (site: citycentremangalore.com)</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>Ask mall marketing/management about weekend kiosk or health-awareness event space. Mall staff and shop owners are also prospects.</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
         <is>
           <t>https://www.uber.com/in/en/blog/places-mlr</t>
         </is>
@@ -4009,20 +4330,25 @@
           <t>Ring Rd, Nijalingappa Layout, Davanagere-Harihara Rd, Davanagere</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K73" s="2" t="inlineStr"/>
-      <c r="L73" s="2" t="inlineStr">
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/studio/body-fuel-fitness-club-davanagere-harihara-road</t>
         </is>
@@ -4057,20 +4383,25 @@
           <t>Kashipur, Shivamogga</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/shimoga/bommanakatte</t>
         </is>
@@ -4105,20 +4436,25 @@
           <t>Vinoba Nagar, Shivamogga</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K75" s="2" t="inlineStr"/>
-      <c r="L75" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/shimoga/bommanakatte</t>
         </is>
@@ -4153,20 +4489,25 @@
           <t>Gandhi Nagar, Shivamogga</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr"/>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K76" s="2" t="inlineStr"/>
-      <c r="L76" s="2" t="inlineStr">
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/shimoga/bommanakatte</t>
         </is>
@@ -4201,20 +4542,25 @@
           <t>Bhadravathi, Shivamogga district</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K77" s="2" t="inlineStr"/>
-      <c r="L77" s="2" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/shimoga/bommanakatte</t>
         </is>
@@ -4249,20 +4595,25 @@
           <t>Sakhar Peth (verify city on Google Maps)</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K78" s="2" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr">
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/kalaburagi</t>
         </is>
@@ -4297,29 +4648,205 @@
           <t>Sakhar Peth (verify city on Google Maps)</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Not found - check Google Maps</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
       <c r="K79" s="2" t="inlineStr"/>
-      <c r="L79" s="2" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr">
         <is>
           <t>https://fitpass.co.in/kalaburagi</t>
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Bellandur / Carmelaram</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Organic store</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Organic Mandya - Bellandur</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Doddakanneli, Carmelaram P.O, Bengaluru 560035</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>+91 96060 01579</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>https://organicmandya.com/collections/organic-mandya-store-in-bellandur</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>HSR Layout</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Organic store</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Organic Mandya - HSR Farmers Market</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>14th Main Rd, opp. Unlimited Fashion, Sector 3, HSR Layout, Bengaluru 560102</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>+91 91084 43222</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>support@organicmandya.com</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Health-conscious shoppers. Ask the owner about putting up a wellness-coaching flyer or doing a weekend awareness stall.</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>https://organicmandya.com/collections/organic-mandya-store-in-bellandur</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Mysuru</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Vijayanagar</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Gold's Gym Mysore Vijaynagar</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>#5658 &amp; 5659, above Style Union, Vijaynagar 2nd Stage, Devraj Mohalla, Mysuru (manager: Prakash)</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>+91 93270 26495</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>jayalakshmipuram.mysore@goldsgym.in (as listed on Gold's Gym site)</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Members want weight-loss / muscle-gain nutrition. Offer a free body-composition check day or a shake counter partnership with the owner/trainers.</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>https://goldsgym.in/our-gyms/gold-s-gym-mysore-vijaynagar/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L79"/>
+  <autoFilter ref="A1:M82"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"New,Called,Visited,Interested,Follow-up,Customer,Not interested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4333,7 +4860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4356,6 +4883,11 @@
           <t>With phone</t>
         </is>
       </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>With email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4364,10 +4896,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C2" t="n">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -4377,9 +4912,12 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4393,7 +4931,10 @@
         <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4408,6 +4949,9 @@
       <c r="C5" t="n">
         <v>1</v>
       </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4421,6 +4965,9 @@
       <c r="C6" t="n">
         <v>0</v>
       </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4434,6 +4981,9 @@
       <c r="C7" t="n">
         <v>0</v>
       </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4447,6 +4997,9 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4460,6 +5013,9 @@
       <c r="C9" t="n">
         <v>0</v>
       </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -4468,10 +5024,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C10" t="n">
-        <v>18</v>
+        <v>26</v>
+      </c>
+      <c r="D10" t="n">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -4485,7 +5044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -4513,86 +5072,93 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EMAILS: small gyms and shops in India rarely publish an email. Only emails actually shown on a public listing are included; none were guessed. For the rest, ask for it on WhatsApp or in person, or check the business's Instagram/Facebook 'Contact' button.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>HERBALIFE RULES TO CHECK FIRST</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Herbalife's distributor rules generally don't allow selling or displaying products in retail stores, malls or supplement shops. Pitch shop/mall owners as personal customers, wellness-event hosts or business-opportunity prospects, not as stockists. Confirm the current rules with your upline or Herbalife India before you start.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Don't make medical or cure claims (e.g. 'cures diabetes'). Talk about nutrition and healthy habits only.</t>
+          <t>Herbalife's distributor rules generally don't allow selling or displaying products in retail stores, malls or supplement shops. Pitch shop/mall owners as personal customers, wellness-event hosts or business-opportunity prospects, not as stockists. Confirm the current rules with your upline or Herbalife India before you start.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Don't make medical or cure claims (e.g. 'cures diabetes'). Talk about nutrition and healthy habits only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>India's TRAI DND rules and the DPDP Act 2023 apply to cold calls and messages. Prefer walk-in visits, ask before adding anyone to WhatsApp groups, and stop if someone says no.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-    </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>WHERE TO FIND MORE LEADS (by hand, free)</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Google Maps: search 'gym in &lt;area&gt;', 'yoga classes in &lt;area&gt;', 'organic store in &lt;area&gt;', 'zumba class in &lt;area&gt;', 'corporate office in &lt;area&gt;'.</t>
+          <t>WHERE TO FIND MORE LEADS (by hand, free)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Justdial / Sulekha / IndiaMART: filter by city and category for phone numbers.</t>
+          <t>Google Maps: search 'gym in &lt;area&gt;', 'yoga classes in &lt;area&gt;', 'organic store in &lt;area&gt;', 'zumba class in &lt;area&gt;', 'corporate office in &lt;area&gt;'.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Smaller cities not yet covered: Tumakuru, Ballari, Vijayapura, Udupi, Hassan, Mandya, Raichur, Bidar, Chitradurga, Hosapete.</t>
+          <t>Justdial / Sulekha / IndiaMART: filter by city and category for phone numbers.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>Smaller cities not yet covered: Tumakuru, Ballari, Vijayapura, Udupi, Hassan, Mandya, Raichur, Bidar, Chitradurga, Hosapete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Other good categories: dance/zumba studios, sports academies, beauty salons and spas, physiotherapy clinics, apartment associations (RWAs), corporate HR wellness teams in IT parks (Manyata, ITPL, Electronic City), college sports departments.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>SIMPLE PROCESS</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>1) Filter the Leads sheet by City. 2) Visit or call 5-10 a day. 3) Update Status and Contacted on. 4) Follow up after 3-7 days with anyone who said Interested.</t>
         </is>

</xml_diff>

<commit_message>
Use Organic Mandya head-office phone for stores without their own number
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GH7UaoDJSnD8fV4SJkmson
</commit_message>
<xml_diff>
--- a/karnataka_herbalife_leads.xlsx
+++ b/karnataka_herbalife_leads.xlsx
@@ -1677,11 +1677,7 @@
           <t>Not found - check Google Maps</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>see rashtrotthana.org</t>
-        </is>
-      </c>
+      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Health-focused members. Pitch a wellness / healthy-breakfast workshop for students.</t>
@@ -2155,7 +2151,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Not found - check Google Maps</t>
+          <t>+91 95909 22000 (Organic Mandya head office)</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2212,7 +2208,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Not found - check Google Maps</t>
+          <t>+91 95909 22000 (Organic Mandya head office)</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2269,7 +2265,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Not found - check Google Maps</t>
+          <t>+91 95909 22000 (Organic Mandya head office)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2326,7 +2322,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Not found - check Google Maps</t>
+          <t>+91 95909 22000 (Organic Mandya head office)</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2383,7 +2379,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Not found - check Google Maps</t>
+          <t>+91 95909 22000 (Organic Mandya head office)</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -4899,10 +4895,10 @@
         <v>41</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -5027,10 +5023,10 @@
         <v>81</v>
       </c>
       <c r="C10" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>